<commit_message>
fix: remove PDF from image-to-pdf accept + vice versa
Auto-swap doesn't make sense for multi-file image tools (jpg-to-pdf,
png-to-pdf accept multiple images to merge into one PDF). Accepting
.pdf there caused broken ZIP downloads.

Auto-swap remains for 1:1 conversion pairs only: PDF↔Word, PDF↔Excel,
PDF↔PPT. These are the tools where users commonly upload the wrong
format.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sofortpdf-google-ads-assets.xlsx
+++ b/sofortpdf-google-ads-assets.xlsx
@@ -2010,7 +2010,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Ab 0,69 € statt 23,99 €/mo</t>
+          <t>PDF-Tools ab nur 0,69 €</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="AJ12" s="2" t="inlineStr">
         <is>
-          <t>Warum 23,99 €/Monat für Adobe zahlen? sofortpdf bietet 19 PDF-Tools ab 0,69 €. Server in der EU. DSGVO-konform.</t>
+          <t>Warum ein teures Adobe-Abo zahlen? sofortpdf bietet 19 PDF-Tools ab 0,69 €. Server in der EU. DSGVO-konform.</t>
         </is>
       </c>
       <c r="AK12" s="2" t="inlineStr">

</xml_diff>